<commit_message>
fix issue#3295, 3294: debook导入issue
</commit_message>
<xml_diff>
--- a/src/assets/template/De-Book Template.xlsx
+++ b/src/assets/template/De-Book Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qyuan4\OneDrive - DXC Production\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GAVIN\PRO_Philips\code_repository\COS-UI\src\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1769060B-3614-4A5E-B387-AAEF0C42A02A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D8C864F-8D32-400B-9775-F95144FDFBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{508F1C01-1DFE-48B5-B5B8-EF954143378D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{508F1C01-1DFE-48B5-B5B8-EF954143378D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,49 +48,49 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{4B9CCD89-3C59-4D3B-A63C-7C9469034ED7}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="F1" authorId="1" shapeId="0" xr:uid="{CFA3A8E2-754B-416A-A7C8-AF3123814806}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     add per requested</t>
       </text>
     </comment>
     <comment ref="H1" authorId="2" shapeId="0" xr:uid="{486F323A-57E4-40DD-AAB4-27B611FE59B7}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="I1" authorId="3" shapeId="0" xr:uid="{22BB3238-075E-4CA5-882B-5647914FB99B}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new add</t>
       </text>
     </comment>
     <comment ref="J1" authorId="4" shapeId="0" xr:uid="{E8557E5F-4FFD-4EE1-9229-3FFE2B8052C3}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new added</t>
       </text>
     </comment>
     <comment ref="K1" authorId="5" shapeId="0" xr:uid="{3572AC16-435B-42E2-A14D-CBC563FC5795}">
       <text>
-        <t>[线程批注]
-你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
-注释:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     new added</t>
       </text>
     </comment>
@@ -107,12 +107,6 @@
     <t>BG(Modality)</t>
   </si>
   <si>
-    <t>销售区域</t>
-  </si>
-  <si>
-    <t xml:space="preserve">销售区域 </t>
-  </si>
-  <si>
     <t>医院编号</t>
   </si>
   <si>
@@ -137,9 +131,6 @@
     <t>进单日期</t>
   </si>
   <si>
-    <t>De-book原因</t>
-  </si>
-  <si>
     <t>Remark</t>
   </si>
   <si>
@@ -288,13 +279,22 @@
   </si>
   <si>
     <t>其他</t>
+  </si>
+  <si>
+    <t>销售区域-team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">销售区域-大区 </t>
+  </si>
+  <si>
+    <t>De-Book原因</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,12 +317,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="宋体"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -399,8 +393,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{D4598283-0CA3-4904-AF18-954A98422C47}"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -443,7 +437,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -773,40 +767,40 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -825,37 +819,37 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$17</xm:f>
           </x14:formula1>
-          <xm:sqref>A1:A1048576</xm:sqref>
+          <xm:sqref>A2:A1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CFC432C-D4BF-431D-B15A-3E8CC5C1D104}">
           <x14:formula1>
             <xm:f>Sheet2!$B$1:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>B1:B1048576</xm:sqref>
+          <xm:sqref>B2:B1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2B19A510-2229-4608-A414-6DD8B1DDF494}">
           <x14:formula1>
             <xm:f>Sheet2!$C$1:$C$21</xm:f>
           </x14:formula1>
-          <xm:sqref>C1:C1048576</xm:sqref>
+          <xm:sqref>C2:C1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3BDD1278-FFAE-4E65-BB9E-7CA5BC99E2B6}">
           <x14:formula1>
             <xm:f>Sheet2!$D$1:$D$16</xm:f>
           </x14:formula1>
-          <xm:sqref>D1:D1048576</xm:sqref>
+          <xm:sqref>D2:D1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{506663EC-6732-4329-9339-13256FAF8A71}">
           <x14:formula1>
             <xm:f>Sheet2!$I$1:$I$2</xm:f>
           </x14:formula1>
-          <xm:sqref>I1:I1048576</xm:sqref>
+          <xm:sqref>I2:I1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E820F090-DBE4-400E-AE43-B61A8064CF3D}">
           <x14:formula1>
             <xm:f>Sheet2!$M$1:$M$7</xm:f>
           </x14:formula1>
-          <xm:sqref>M1:M1048576</xm:sqref>
+          <xm:sqref>M2:M1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -870,242 +864,242 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="C18" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="C19" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="C20" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="C21" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>